<commit_message>
Enrich sample Excel files to 8-11 tasks per epic
Each workstream file now has 8-11 realistic, properly dated tasks per
epic covering design, build, test, UAT and sign-off phases. ZIP files
rebuilt to include the enriched data.

https://claude.ai/code/session_01YJLCQM1jYoVm9fLznkPWBk
</commit_message>
<xml_diff>
--- a/samples/sample1/Card_Payments.xlsx
+++ b/samples/sample1/Card_Payments.xlsx
@@ -66,9 +66,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -663,9 +664,560 @@
         <v>46204</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>CP-09</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Card scheme registration &amp; BIN allocation</v>
+      </c>
+      <c r="E11" t="str">
+        <v>1</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G11" t="str">
+        <v>100</v>
+      </c>
+      <c r="H11" s="2">
+        <v>46096</v>
+      </c>
+      <c r="I11" s="2">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>CP-10</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Embossing &amp; personalisation vendor setup</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G12" t="str">
+        <v>85</v>
+      </c>
+      <c r="H12" s="2">
+        <v>46113</v>
+      </c>
+      <c r="I12" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>CP-11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D13" t="str">
+        <v>PIN management system integration</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G13" t="str">
+        <v>60</v>
+      </c>
+      <c r="H13" s="2">
+        <v>46141</v>
+      </c>
+      <c r="I13" s="2">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>CP-12</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Cardholder agreement &amp; T&amp;Cs</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Governance</v>
+      </c>
+      <c r="G14" t="str">
+        <v>55</v>
+      </c>
+      <c r="H14" s="2">
+        <v>46155</v>
+      </c>
+      <c r="I14" s="2">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>CP-13</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Card activation &amp; lifecycle workflow</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G15" t="str">
+        <v>30</v>
+      </c>
+      <c r="H15" s="2">
+        <v>46169</v>
+      </c>
+      <c r="I15" s="2">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CP-14</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Issuing</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Issuing UAT &amp; scheme certification</v>
+      </c>
+      <c r="E16" t="str">
+        <v>1</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Testing</v>
+      </c>
+      <c r="G16" t="str">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>46190</v>
+      </c>
+      <c r="I16" s="2">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>CP-15</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Merchant agreement &amp; onboarding template</v>
+      </c>
+      <c r="E17" t="str">
+        <v>1</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G17" t="str">
+        <v>100</v>
+      </c>
+      <c r="H17" s="2">
+        <v>46113</v>
+      </c>
+      <c r="I17" s="2">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>CP-16</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D18" t="str">
+        <v>POS terminal deployment plan</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G18" t="str">
+        <v>80</v>
+      </c>
+      <c r="H18" s="2">
+        <v>46127</v>
+      </c>
+      <c r="I18" s="2">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>CP-17</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Settlement &amp; reconciliation design</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Payments</v>
+      </c>
+      <c r="G19" t="str">
+        <v>60</v>
+      </c>
+      <c r="H19" s="2">
+        <v>46148</v>
+      </c>
+      <c r="I19" s="2">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>CP-18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Chargeback &amp; dispute workflow</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G20" t="str">
+        <v>35</v>
+      </c>
+      <c r="H20" s="2">
+        <v>46169</v>
+      </c>
+      <c r="I20" s="2">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>CP-19</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D21" t="str">
+        <v>PCI-DSS compliance verification</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Security</v>
+      </c>
+      <c r="G21" t="str">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2">
+        <v>46176</v>
+      </c>
+      <c r="I21" s="2">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>CP-20</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Acquiring</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Acquiring UAT &amp; scheme certification</v>
+      </c>
+      <c r="E22" t="str">
+        <v>1</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Testing</v>
+      </c>
+      <c r="G22" t="str">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2">
+        <v>46204</v>
+      </c>
+      <c r="I22" s="2">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>CP-21</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Fraud strategy &amp; rules design</v>
+      </c>
+      <c r="E23" t="str">
+        <v>1</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G23" t="str">
+        <v>100</v>
+      </c>
+      <c r="H23" s="2">
+        <v>46113</v>
+      </c>
+      <c r="I23" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>CP-22</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Real-time scoring model integration</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G24" t="str">
+        <v>70</v>
+      </c>
+      <c r="H24" s="2">
+        <v>46134</v>
+      </c>
+      <c r="I24" s="2">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>CP-23</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D25" t="str">
+        <v>3DS2 challenge &amp; exemptions config</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G25" t="str">
+        <v>55</v>
+      </c>
+      <c r="H25" s="2">
+        <v>46155</v>
+      </c>
+      <c r="I25" s="2">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>CP-24</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Fraud alert &amp; case management setup</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G26" t="str">
+        <v>30</v>
+      </c>
+      <c r="H26" s="2">
+        <v>46169</v>
+      </c>
+      <c r="I26" s="2">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>CP-25</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Fraud analytics dashboard</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G27" t="str">
+        <v>10</v>
+      </c>
+      <c r="H27" s="2">
+        <v>46190</v>
+      </c>
+      <c r="I27" s="2">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>CP-26</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Regulatory fraud reporting</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Compliance</v>
+      </c>
+      <c r="G28" t="str">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <v>46204</v>
+      </c>
+      <c r="I28" s="2">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>CP-27</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Card Payments</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Fraud</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Fraud UAT &amp; model tuning</v>
+      </c>
+      <c r="E29" t="str">
+        <v>1</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Testing</v>
+      </c>
+      <c r="G29" t="str">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <v>46211</v>
+      </c>
+      <c r="I29" s="2">
+        <v>46232</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>